<commit_message>
add notes for rects
</commit_message>
<xml_diff>
--- a/docs/notes.xlsx
+++ b/docs/notes.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nkiser\Documents\Pebble_Fresco\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E490CC47-0E55-4E0F-893A-0F03863BCE8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D35F46FD-8436-4EE9-92EF-9557091E009D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="720" windowWidth="14235" windowHeight="15480" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="time_text" sheetId="1" r:id="rId1"/>
+    <sheet name="rectangles" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="251">
   <si>
     <t>X:00</t>
   </si>
@@ -293,9 +294,6 @@
     <t>J</t>
   </si>
   <si>
-    <t>word one</t>
-  </si>
-  <si>
     <t>X:22</t>
   </si>
   <si>
@@ -314,9 +312,6 @@
     <t>K</t>
   </si>
   <si>
-    <t>word two</t>
-  </si>
-  <si>
     <t>X:24</t>
   </si>
   <si>
@@ -329,9 +324,6 @@
     <t>L</t>
   </si>
   <si>
-    <t>word three</t>
-  </si>
-  <si>
     <t>X:26</t>
   </si>
   <si>
@@ -374,9 +366,6 @@
     <t>N</t>
   </si>
   <si>
-    <t>0-23, no leading space</t>
-  </si>
-  <si>
     <t>X:30</t>
   </si>
   <si>
@@ -386,9 +375,6 @@
     <t>o</t>
   </si>
   <si>
-    <t>1-12, no leading space</t>
-  </si>
-  <si>
     <t>X:31</t>
   </si>
   <si>
@@ -521,9 +507,6 @@
     <t>v</t>
   </si>
   <si>
-    <t>current steps</t>
-  </si>
-  <si>
     <t>X:45</t>
   </si>
   <si>
@@ -596,17 +579,224 @@
     <t>X:59</t>
   </si>
   <si>
-    <t>watch-settings 01-12 or 00-23</t>
-  </si>
-  <si>
-    <t>watch-settings 1-12 or 00-23</t>
+    <t>Radius</t>
+  </si>
+  <si>
+    <t>Outline</t>
+  </si>
+  <si>
+    <t>Dither</t>
+  </si>
+  <si>
+    <t>int</t>
+  </si>
+  <si>
+    <t>bool</t>
+  </si>
+  <si>
+    <t>UD/LR/MIX</t>
+  </si>
+  <si>
+    <t>Foreground</t>
+  </si>
+  <si>
+    <t>Background</t>
+  </si>
+  <si>
+    <t>Color</t>
+  </si>
+  <si>
+    <t>Inverter</t>
+  </si>
+  <si>
+    <t>Font Family</t>
+  </si>
+  <si>
+    <t>Word-Wrap</t>
+  </si>
+  <si>
+    <t>1 to 31</t>
+  </si>
+  <si>
+    <t>uint</t>
+  </si>
+  <si>
+    <t>Alignment</t>
+  </si>
+  <si>
+    <t>L-C-R</t>
+  </si>
+  <si>
+    <t>If text:</t>
+  </si>
+  <si>
+    <t>All rect's</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If not text </t>
+  </si>
+  <si>
+    <t>and Dyn Size</t>
+  </si>
+  <si>
+    <t>Param:</t>
+  </si>
+  <si>
+    <t>Divisor</t>
+  </si>
+  <si>
+    <t>Addend</t>
+  </si>
+  <si>
+    <t>Monday</t>
+  </si>
+  <si>
+    <t>Jan</t>
+  </si>
+  <si>
+    <t>Mon</t>
+  </si>
+  <si>
+    <t>Janurary</t>
+  </si>
+  <si>
+    <t>Day of Month 01-31</t>
+  </si>
+  <si>
+    <t>mm/dd/yy</t>
+  </si>
+  <si>
+    <t>hour 0-23, no leading space</t>
+  </si>
+  <si>
+    <t>hour 1-12, no leading space</t>
+  </si>
+  <si>
+    <t>day of month 1-31, w/ leading space 1-9</t>
+  </si>
+  <si>
+    <t>"modifier"</t>
+  </si>
+  <si>
+    <t>ISO 8601 Date YYYY-mm-dd</t>
+  </si>
+  <si>
+    <t>ISO 8601 week-based year (not YYYY)</t>
+  </si>
+  <si>
+    <t>ISO 8601 week-based year no century (not yy)</t>
+  </si>
+  <si>
+    <t>Century 19-20 (2026-&gt; 20)</t>
+  </si>
+  <si>
+    <t>hour 00-23</t>
+  </si>
+  <si>
+    <t>hour 01-12</t>
+  </si>
+  <si>
+    <t>day of year 001-366</t>
+  </si>
+  <si>
+    <t>3-word time: word one</t>
+  </si>
+  <si>
+    <t>3-word time: word two</t>
+  </si>
+  <si>
+    <t>3-word time: word three</t>
+  </si>
+  <si>
+    <t>hour 0-23, w/ leading space 0-9</t>
+  </si>
+  <si>
+    <t>hour 1-12, w/ leading space 1-9</t>
+  </si>
+  <si>
+    <t>month 01-12</t>
+  </si>
+  <si>
+    <t>minute 0-59</t>
+  </si>
+  <si>
+    <t>AM/PM</t>
+  </si>
+  <si>
+    <t>am/pm</t>
+  </si>
+  <si>
+    <t>watch-settings 1-12 or 00-23 (no leading space)</t>
+  </si>
+  <si>
+    <t>watch-settings 01-12 or 00-23 (leading zero)</t>
+  </si>
+  <si>
+    <t>24-hr time "15:31"</t>
+  </si>
+  <si>
+    <t>am/pm time "03:31:59 pm"</t>
+  </si>
+  <si>
+    <t>24-hr time "15:31:59"</t>
+  </si>
+  <si>
+    <t>tab character</t>
+  </si>
+  <si>
+    <t>newline character</t>
+  </si>
+  <si>
+    <t>seconds 00-59</t>
+  </si>
+  <si>
+    <t>seconds since epoch (1970-01-01 00:00:00)</t>
+  </si>
+  <si>
+    <t>day of week, Monday=1, 1-7</t>
+  </si>
+  <si>
+    <t>day of week, Sunday=0, 0-6</t>
+  </si>
+  <si>
+    <t>week number 00-53, starting with the first Sunday as first day of week 01</t>
+  </si>
+  <si>
+    <t>ISO 8601 week number 01-53, week 1 is first week w/ 4+ days</t>
+  </si>
+  <si>
+    <t>week number 00-53, starting with the first Monday as first day of week 01</t>
+  </si>
+  <si>
+    <t>locale date (in US, mm/dd/yy)</t>
+  </si>
+  <si>
+    <t>locale date and time (in US, Mon Jan 05 15:31:59 2026)</t>
+  </si>
+  <si>
+    <t>locale time (in US, 15:31:59)</t>
+  </si>
+  <si>
+    <t>2-digit year 00-99</t>
+  </si>
+  <si>
+    <t>4-digit year</t>
+  </si>
+  <si>
+    <t>+hhmm or -hhmm timezone offsetrom UTC</t>
+  </si>
+  <si>
+    <t>timezone name or abbreviation</t>
+  </si>
+  <si>
+    <t>today's steps</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -621,8 +811,22 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -635,6 +839,16 @@
         <bgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -645,17 +859,26 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="3" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="4">
+    <cellStyle name="Bad" xfId="3" builtinId="27"/>
     <cellStyle name="Excel Built-in Neutral" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="Good" xfId="2" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -975,6 +1198,9 @@
       <c r="O3" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="P3" t="s">
+        <v>205</v>
+      </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -995,6 +1221,9 @@
       <c r="O4" s="1" t="s">
         <v>16</v>
       </c>
+      <c r="P4" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
@@ -1015,6 +1244,9 @@
       <c r="O5" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="P5" t="s">
+        <v>204</v>
+      </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -1046,6 +1278,9 @@
       <c r="O6" s="1" t="s">
         <v>23</v>
       </c>
+      <c r="P6" t="s">
+        <v>206</v>
+      </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -1077,6 +1312,9 @@
       <c r="O7" s="1" t="s">
         <v>26</v>
       </c>
+      <c r="P7" t="s">
+        <v>244</v>
+      </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -1094,6 +1332,9 @@
       <c r="O8" s="1" t="s">
         <v>29</v>
       </c>
+      <c r="P8" t="s">
+        <v>216</v>
+      </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
@@ -1125,6 +1366,9 @@
       <c r="O9" s="1" t="s">
         <v>32</v>
       </c>
+      <c r="P9" t="s">
+        <v>207</v>
+      </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -1142,6 +1386,9 @@
       <c r="O10" s="1" t="s">
         <v>35</v>
       </c>
+      <c r="P10" t="s">
+        <v>208</v>
+      </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
@@ -1176,6 +1423,9 @@
       <c r="O11" s="1" t="s">
         <v>41</v>
       </c>
+      <c r="P11" t="s">
+        <v>211</v>
+      </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -1206,8 +1456,11 @@
         <f>G12*4/16</f>
         <v>804</v>
       </c>
-      <c r="O12" s="1" t="s">
+      <c r="O12" s="4" t="s">
         <v>44</v>
+      </c>
+      <c r="P12" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
@@ -1238,7 +1491,7 @@
         <f>4.5*256</f>
         <v>1152</v>
       </c>
-      <c r="O13" t="s">
+      <c r="O13" s="5" t="s">
         <v>47</v>
       </c>
       <c r="P13" t="s">
@@ -1265,6 +1518,9 @@
       <c r="O14" s="1" t="s">
         <v>51</v>
       </c>
+      <c r="P14" t="s">
+        <v>213</v>
+      </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -1290,6 +1546,9 @@
       <c r="O15" s="1" t="s">
         <v>55</v>
       </c>
+      <c r="P15" t="s">
+        <v>215</v>
+      </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
@@ -1311,6 +1570,9 @@
       <c r="O16" s="1" t="s">
         <v>58</v>
       </c>
+      <c r="P16" t="s">
+        <v>214</v>
+      </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -1328,6 +1590,9 @@
       <c r="O17" s="1" t="s">
         <v>61</v>
       </c>
+      <c r="P17" t="s">
+        <v>204</v>
+      </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
@@ -1357,6 +1622,9 @@
       <c r="O18" s="1" t="s">
         <v>67</v>
       </c>
+      <c r="P18" t="s">
+        <v>217</v>
+      </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
@@ -1387,8 +1655,11 @@
       <c r="I19" t="s">
         <v>71</v>
       </c>
-      <c r="O19" t="s">
+      <c r="O19" s="5" t="s">
         <v>72</v>
+      </c>
+      <c r="P19" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
@@ -1423,6 +1694,9 @@
       <c r="O20" s="1" t="s">
         <v>77</v>
       </c>
+      <c r="P20" t="s">
+        <v>218</v>
+      </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
@@ -1456,6 +1730,9 @@
       <c r="O21" s="1" t="s">
         <v>81</v>
       </c>
+      <c r="P21" t="s">
+        <v>219</v>
+      </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
@@ -1486,16 +1763,16 @@
       <c r="I22" t="s">
         <v>83</v>
       </c>
-      <c r="O22" t="s">
+      <c r="O22" s="5" t="s">
         <v>84</v>
       </c>
       <c r="P22" t="s">
-        <v>85</v>
+        <v>220</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B23" t="s">
         <v>1</v>
@@ -1520,15 +1797,18 @@
         <v>32.400000000000006</v>
       </c>
       <c r="I23" t="s">
+        <v>86</v>
+      </c>
+      <c r="O23" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="O23" s="1" t="s">
-        <v>88</v>
+      <c r="P23" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B24" t="s">
         <v>1</v>
@@ -1553,18 +1833,18 @@
         <v>32.400000000000006</v>
       </c>
       <c r="I24" t="s">
+        <v>89</v>
+      </c>
+      <c r="O24" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="O24" t="s">
-        <v>91</v>
-      </c>
       <c r="P24" t="s">
-        <v>92</v>
+        <v>221</v>
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B25" t="s">
         <v>1</v>
@@ -1579,7 +1859,7 @@
         <v>7</v>
       </c>
       <c r="F25" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G25">
         <v>28</v>
@@ -1589,12 +1869,15 @@
         <v>37.800000000000004</v>
       </c>
       <c r="O25" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
+      </c>
+      <c r="P25" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B26" t="s">
         <v>1</v>
@@ -1609,7 +1892,7 @@
         <v>8</v>
       </c>
       <c r="F26" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G26">
         <v>28</v>
@@ -1618,16 +1901,16 @@
         <f t="shared" si="0"/>
         <v>37.800000000000004</v>
       </c>
-      <c r="O26" t="s">
-        <v>96</v>
+      <c r="O26" s="5" t="s">
+        <v>94</v>
       </c>
       <c r="P26" t="s">
-        <v>97</v>
+        <v>222</v>
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B27" t="s">
         <v>1</v>
@@ -1642,7 +1925,7 @@
         <v>9</v>
       </c>
       <c r="F27" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G27">
         <v>30</v>
@@ -1652,15 +1935,18 @@
         <v>40.5</v>
       </c>
       <c r="I27" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="O27" s="1" t="s">
-        <v>101</v>
+        <v>98</v>
+      </c>
+      <c r="P27" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B28" t="s">
         <v>1</v>
@@ -1675,7 +1961,7 @@
         <v>10</v>
       </c>
       <c r="F28" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="G28">
         <v>34</v>
@@ -1685,15 +1971,18 @@
         <v>45.900000000000006</v>
       </c>
       <c r="I28" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="O28" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
+      </c>
+      <c r="P28" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B29" t="s">
         <v>1</v>
@@ -1708,7 +1997,7 @@
         <v>11</v>
       </c>
       <c r="F29" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="G29">
         <v>42</v>
@@ -1718,15 +2007,18 @@
         <v>56.7</v>
       </c>
       <c r="I29" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="O29" s="1" t="s">
-        <v>108</v>
+        <v>105</v>
+      </c>
+      <c r="P29" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B30" t="s">
         <v>1</v>
@@ -1741,7 +2033,7 @@
         <v>12</v>
       </c>
       <c r="F30" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="G30">
         <v>42</v>
@@ -1751,21 +2043,21 @@
         <v>56.7</v>
       </c>
       <c r="I30" t="s">
-        <v>107</v>
-      </c>
-      <c r="O30" t="s">
-        <v>111</v>
+        <v>104</v>
+      </c>
+      <c r="O30" s="5" t="s">
+        <v>108</v>
       </c>
       <c r="P30" t="s">
-        <v>112</v>
+        <v>209</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B31" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C31" t="s">
         <v>22</v>
@@ -1777,7 +2069,7 @@
         <v>13</v>
       </c>
       <c r="F31" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="G31">
         <v>42</v>
@@ -1787,24 +2079,24 @@
         <v>56.7</v>
       </c>
       <c r="I31" t="s">
-        <v>107</v>
-      </c>
-      <c r="O31" t="s">
-        <v>115</v>
+        <v>104</v>
+      </c>
+      <c r="O31" s="5" t="s">
+        <v>111</v>
       </c>
       <c r="P31" t="s">
-        <v>116</v>
+        <v>210</v>
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B32" t="s">
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="D32" t="s">
         <v>6</v>
@@ -1813,7 +2105,7 @@
         <v>14</v>
       </c>
       <c r="F32" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="G32">
         <v>21</v>
@@ -1823,21 +2115,24 @@
         <v>28.35</v>
       </c>
       <c r="I32" t="s">
-        <v>87</v>
-      </c>
-      <c r="O32" s="1" t="s">
-        <v>120</v>
+        <v>86</v>
+      </c>
+      <c r="O32" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="P32" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B33" t="s">
         <v>1</v>
       </c>
       <c r="C33" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="D33" t="s">
         <v>10</v>
@@ -1846,7 +2141,7 @@
         <v>15</v>
       </c>
       <c r="F33" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="G33">
         <v>49</v>
@@ -1856,18 +2151,21 @@
         <v>66.150000000000006</v>
       </c>
       <c r="O33" s="1" t="s">
-        <v>122</v>
+        <v>117</v>
+      </c>
+      <c r="P33" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B34" t="s">
         <v>1</v>
       </c>
       <c r="C34" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="D34" t="s">
         <v>14</v>
@@ -1876,7 +2174,7 @@
         <v>16</v>
       </c>
       <c r="F34" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="G34">
         <v>28</v>
@@ -1886,18 +2184,21 @@
         <v>37.800000000000004</v>
       </c>
       <c r="O34" s="1" t="s">
-        <v>125</v>
+        <v>120</v>
+      </c>
+      <c r="P34" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B35" t="s">
         <v>1</v>
       </c>
       <c r="C35" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="D35" t="s">
         <v>18</v>
@@ -1906,7 +2207,7 @@
         <v>17</v>
       </c>
       <c r="F35" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="G35">
         <v>20</v>
@@ -1916,24 +2217,24 @@
         <v>27</v>
       </c>
       <c r="I35" t="s">
-        <v>128</v>
-      </c>
-      <c r="O35" t="s">
-        <v>129</v>
+        <v>123</v>
+      </c>
+      <c r="O35" s="5" t="s">
+        <v>124</v>
       </c>
       <c r="P35" t="s">
-        <v>186</v>
+        <v>230</v>
       </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="B36" t="s">
         <v>1</v>
       </c>
       <c r="C36" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="D36" t="s">
         <v>21</v>
@@ -1942,7 +2243,7 @@
         <v>18</v>
       </c>
       <c r="F36" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="G36">
         <v>26</v>
@@ -1952,24 +2253,24 @@
         <v>35.1</v>
       </c>
       <c r="I36" t="s">
-        <v>131</v>
-      </c>
-      <c r="O36" t="s">
-        <v>132</v>
+        <v>126</v>
+      </c>
+      <c r="O36" s="5" t="s">
+        <v>127</v>
       </c>
       <c r="P36" t="s">
-        <v>187</v>
+        <v>229</v>
       </c>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="B37" t="s">
         <v>1</v>
       </c>
       <c r="C37" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="D37" t="s">
         <v>25</v>
@@ -1978,7 +2279,7 @@
         <v>19</v>
       </c>
       <c r="F37" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="G37">
         <v>28</v>
@@ -1988,21 +2289,24 @@
         <v>37.800000000000004</v>
       </c>
       <c r="I37" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="O37" s="1" t="s">
-        <v>135</v>
+        <v>130</v>
+      </c>
+      <c r="P37" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="B38" t="s">
         <v>1</v>
       </c>
       <c r="C38" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="D38" t="s">
         <v>28</v>
@@ -2011,7 +2315,7 @@
         <v>20</v>
       </c>
       <c r="F38" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="G38">
         <v>32</v>
@@ -2021,21 +2325,24 @@
         <v>43.2</v>
       </c>
       <c r="I38" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="O38" s="1" t="s">
-        <v>138</v>
+        <v>133</v>
+      </c>
+      <c r="P38" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="B39" t="s">
         <v>1</v>
       </c>
       <c r="C39" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="D39" t="s">
         <v>31</v>
@@ -2044,7 +2351,7 @@
         <v>21</v>
       </c>
       <c r="F39" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="G39">
         <v>36</v>
@@ -2054,21 +2361,24 @@
         <v>48.6</v>
       </c>
       <c r="I39" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="O39" s="1" t="s">
-        <v>141</v>
+        <v>136</v>
+      </c>
+      <c r="P39" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="B40" t="s">
         <v>1</v>
       </c>
       <c r="C40" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="D40" t="s">
         <v>34</v>
@@ -2077,7 +2387,7 @@
         <v>22</v>
       </c>
       <c r="F40" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="G40">
         <v>38</v>
@@ -2087,30 +2397,33 @@
         <v>51.300000000000004</v>
       </c>
       <c r="I40" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="O40" s="1" t="s">
-        <v>144</v>
+        <v>139</v>
+      </c>
+      <c r="P40" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="B41" t="s">
         <v>79</v>
       </c>
       <c r="C41" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="D41" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="E41">
         <v>23</v>
       </c>
       <c r="F41" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="G41">
         <v>42</v>
@@ -2120,21 +2433,24 @@
         <v>56.7</v>
       </c>
       <c r="I41" t="s">
+        <v>138</v>
+      </c>
+      <c r="O41" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="O41" s="1" t="s">
-        <v>148</v>
+      <c r="P41" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="B42" t="s">
         <v>1</v>
       </c>
       <c r="C42" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="D42" t="s">
         <v>6</v>
@@ -2143,7 +2459,7 @@
         <v>24</v>
       </c>
       <c r="F42" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="G42">
         <v>60</v>
@@ -2153,18 +2469,21 @@
         <v>81</v>
       </c>
       <c r="O42" s="1" t="s">
-        <v>152</v>
+        <v>147</v>
+      </c>
+      <c r="P42" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="B43" t="s">
         <v>1</v>
       </c>
       <c r="C43" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="D43" t="s">
         <v>10</v>
@@ -2173,7 +2492,7 @@
         <v>25</v>
       </c>
       <c r="F43" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="G43">
         <v>60</v>
@@ -2182,110 +2501,122 @@
         <f t="shared" si="0"/>
         <v>81</v>
       </c>
-      <c r="O43" t="s">
-        <v>155</v>
+      <c r="O43" s="7" t="s">
+        <v>150</v>
       </c>
       <c r="P43" t="s">
-        <v>156</v>
+        <v>238</v>
       </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="B44" t="s">
         <v>1</v>
       </c>
       <c r="C44" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="D44" t="s">
         <v>14</v>
       </c>
       <c r="O44" s="1" t="s">
-        <v>158</v>
+        <v>153</v>
+      </c>
+      <c r="P44" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="B45" t="s">
         <v>1</v>
       </c>
       <c r="C45" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="D45" t="s">
         <v>18</v>
       </c>
-      <c r="O45" t="s">
-        <v>160</v>
+      <c r="O45" s="5" t="s">
+        <v>155</v>
       </c>
       <c r="P45" t="s">
-        <v>161</v>
+        <v>250</v>
       </c>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="B46" t="s">
         <v>57</v>
       </c>
       <c r="C46" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="D46" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="O46" s="1" t="s">
-        <v>163</v>
+        <v>157</v>
+      </c>
+      <c r="P46" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="B47" t="s">
         <v>1</v>
       </c>
       <c r="C47" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="D47" t="s">
         <v>25</v>
       </c>
       <c r="O47" s="1" t="s">
-        <v>165</v>
+        <v>159</v>
+      </c>
+      <c r="P47" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="B48" t="s">
         <v>1</v>
       </c>
       <c r="C48" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="D48" t="s">
         <v>28</v>
       </c>
       <c r="O48" s="1" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+        <v>161</v>
+      </c>
+      <c r="P48" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="B49" t="s">
         <v>1</v>
       </c>
       <c r="C49" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="D49" t="s">
         <v>31</v>
@@ -2293,171 +2624,189 @@
       <c r="O49" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P49" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="B50" t="s">
         <v>1</v>
       </c>
       <c r="C50" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="D50" t="s">
         <v>34</v>
       </c>
       <c r="O50" s="1" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
+        <v>164</v>
+      </c>
+      <c r="P50" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="B51" t="s">
         <v>37</v>
       </c>
       <c r="C51" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="D51" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="O51" s="1" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
+        <v>166</v>
+      </c>
+      <c r="P51" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="B52" t="s">
         <v>1</v>
       </c>
       <c r="C52" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="D52" t="s">
         <v>6</v>
       </c>
       <c r="O52" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+        <v>169</v>
+      </c>
+      <c r="P52" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="B53" t="s">
         <v>1</v>
       </c>
       <c r="C53" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="D53" t="s">
         <v>10</v>
       </c>
       <c r="O53" s="1" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
+        <v>171</v>
+      </c>
+      <c r="P53" s="6" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="B54" t="s">
         <v>1</v>
       </c>
       <c r="C54" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="D54" t="s">
         <v>14</v>
       </c>
       <c r="O54" s="1" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
+        <v>173</v>
+      </c>
+      <c r="P54" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="B55" t="s">
         <v>1</v>
       </c>
       <c r="C55" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="D55" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="B56" t="s">
         <v>21</v>
       </c>
       <c r="C56" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="D56" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="B57" t="s">
         <v>1</v>
       </c>
       <c r="C57" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="D57" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="B58" t="s">
         <v>1</v>
       </c>
       <c r="C58" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="D58" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="B59" t="s">
         <v>1</v>
       </c>
       <c r="C59" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="D59" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="B60" t="s">
         <v>1</v>
       </c>
       <c r="C60" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="D60" t="s">
         <v>34</v>
@@ -2467,4 +2816,156 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A50F46B-BD0C-4AF8-9BB8-27411F685027}">
+  <dimension ref="A1:C19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1" t="s">
+        <v>164</v>
+      </c>
+      <c r="C1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>161</v>
+      </c>
+      <c r="C3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C4" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>180</v>
+      </c>
+      <c r="C5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>181</v>
+      </c>
+      <c r="C6" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>182</v>
+      </c>
+      <c r="C7" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>186</v>
+      </c>
+      <c r="C8" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>187</v>
+      </c>
+      <c r="C9" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>189</v>
+      </c>
+      <c r="C10" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>196</v>
+      </c>
+      <c r="B12" t="s">
+        <v>190</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>191</v>
+      </c>
+      <c r="C13" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>194</v>
+      </c>
+      <c r="C14" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>199</v>
+      </c>
+      <c r="B16" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>201</v>
+      </c>
+      <c r="C18" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
+        <v>202</v>
+      </c>
+      <c r="C19" t="s">
+        <v>193</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>